<commit_message>
Route borrower visitors to the borrower pilot form; refresh social previews
- The borrower demo's pilot link carries workflow=assess, and the pilot page's
  sidebar and demo link follow the selected workflow.
- Homepage title, description and Open Graph/Twitter tags describe both
  workflows; the preview image is now a 1200x630 PNG (WhatsApp does not
  render SVG previews).
- Retention is described everywhere as credits matched by subsequent debits,
  a timing pattern rather than money traced; demo snapshot re-exported.
</commit_message>
<xml_diff>
--- a/static/demo/assess/case_76.xlsx
+++ b/static/demo/assess/case_76.xlsx
@@ -3856,7 +3856,7 @@
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>Large credits moved out within 2 days (share)</t>
+          <t>Credits matched by subsequent debits within 2 days (share of large credits)</t>
         </is>
       </c>
       <c r="B31" s="9" t="n">
@@ -4564,7 +4564,7 @@
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>Large credits moved out within 2 days (share)</t>
+          <t>Credits matched by subsequent debits within 2 days (share of large credits)</t>
         </is>
       </c>
       <c r="B65" s="9" t="n">

</xml_diff>